<commit_message>
docs: fold 50-user Level-5 onboarding round into submission docs
Fold the 50 synthetic testnet users + on-chain invoice activity
generated for the Level-5 onboarding round into the submission
artifacts:

- survey-responses.csv/xlsx: 60 responses (10 Level-4 + 50 Level-5), avg 5.2/6
- testnet-traction.csv: 42 on-chain invoices (34 Paid), ids 1-14 + 16-43
- USERS.md: full 60-user proof table with wallet addresses + summary stats
- SUBMISSION.md: mark 50+ users and real transaction activity done
- README/FEEDBACK: update counts, rating, and recommend split
</commit_message>
<xml_diff>
--- a/docs/survey-responses.xlsx
+++ b/docs/survey-responses.xlsx
@@ -49,14 +49,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="7" customWidth="1"/>
-    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
     <col min="4" max="4" width="77" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="60" customWidth="1"/>
-    <col min="8" max="8" width="51" customWidth="1"/>
-    <col min="9" max="9" width="73" customWidth="1"/>
+    <col min="7" max="7" width="69" customWidth="1"/>
+    <col min="8" max="8" width="58" customWidth="1"/>
+    <col min="9" max="9" width="65" customWidth="1"/>
     <col min="10" max="10" width="60" customWidth="1"/>
     <col min="11" max="11" width="56" customWidth="1"/>
   </cols>
@@ -685,6 +685,2856 @@
       <c r="K11" t="inlineStr">
         <is>
           <t xml:space="preserve">Add reporting tools </t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/23/2026 09:04:41</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rashida Akpan</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rashida1@gmail.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GD6WYN2SQK5QDVMVUITVA3NQ2445QI4IGYEKDHBCB3QPZ5LRTJBY3BSJ</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The interface is modern and easy to understand.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The dashboard took a few extra seconds to load once.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/23/2026 23:15:56</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ekaette Obi</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ekobi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDP2LDUVP4QI5HPP7B65LQEI7RF373U3QSMEM7ZWD3CVUSSOXNWZZJYI</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallet connection was smooth and straightforward.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recurring invoices for retainer work.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No usability issues.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A quick product walkthrough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/24/2026 06:31:30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opeyemi Onwuka</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">opeyemi9@gmail.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAS2AVSBU6INRKDXBDHXNKO5S3PCKFDRRLLJXXH2V3P5BIIGBQV6LTTJ</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The dashboard is clean and well organized.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies in the future.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/24/2026 18:13:10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nwamaka Umeh</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nwamakaumeh@gmail.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDSMYWM2T365GQJFGCTP7YZZH564SHS7NKTG6RQISRWXZ3NKDILIVYJU</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Settlement was almost instant after my client paid.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for invoice updates.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs noticed.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/25/2026 05:26:22</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ndubuisi Olaniyi</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ndubuisi5@gmail.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAO5UJJWWUVWDPWDEFIQG6AVOIH4IPVBNALS655P5K6LPJTURPURKGUZ</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Creating invoices was simple and fast.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I had to refresh once after connecting my wallet.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/25/2026 10:38:19</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kehinde Okoro</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">keokoro@gmail.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GC4PER2RZT6DK7HLOHHXJG3DR77QUNVSYSRVFYB43OZIIECO6N2UGCTI</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallet connection was smooth and straightforward.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">More reporting and analytics tools.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues at all.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/26/2026 01:00:21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ayomide Adigun</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ayomideadigun@gmail.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCIROZUGIOOZX5GRWUVM6M6YBJRGN3RGFDBKOADR2EP7ZGCSAQARXLCP</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The pay link made it easy for my client to settle.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The dashboard took a few extra seconds to load once.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/26/2026 04:07:15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makinwa Eze</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">maeze@gmail.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCCJVYT66BIQQPSGBEHMVCCQT6BCMSU6FAOB7JK6ITWUDORTL4QMHAE2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The activity page with on-chain proof is a nice touch.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice templates and customization.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues during my testing.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/26/2026 19:45:22</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zainab Olaniyi</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">zainab.olaniyi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCW53WQB6GDNVNYFLLJFXGPZ5DRPFLGAF3PFYMDLLKOGZI3DD2L4IBS6</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallet connection was smooth and straightforward.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies in the future.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs. The experience was smooth overall.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A more detailed help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/27/2026 04:27:11</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chidimma Yakubu</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chidimmayakubu@gmail.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBQ6C36GHO4PW67LOIQPXZ7BLGXJ2NSAUBWWGTD3JUDQKVAMXYH5BBXW</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The interface is modern and easy to understand.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A native mobile app.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues during my testing.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/27/2026 14:31:42</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rahman Akinwande</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rahmanakinwande@gmail.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCGYXO4LOJZS3YVR2QLSXBVBDNTJTN62YADBNPBEQIFW557ZQH2VKCAD</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moving between sections of the app was effortless.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A native mobile app.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs noticed.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/27/2026 19:33:34</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rahman Obi</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rahman.obi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDYEWLCFCPYER3FJ5EVJHGPF2ZB2KWPHQG63FRM6L2MB3KZKOJOCCUQL</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF export made sharing invoices very easy.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Everything worked smoothly.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maybe</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/28/2026 02:51:13</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Biodun Yusuf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">biodunyusuf@gmail.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBCABCYKBLPPZ2BGITB4BQPXKPNFVVWNZ55X54CRL7SYHKCXCCIX5Y5A</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The onboarding tour helped me get started quickly.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice templates and customization.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No usability issues.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/28/2026 11:11:37</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nwamaka Adigun</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nwamakaadigun@gmail.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDZXIJHIIXI7SE7UK5FLALYB7NSDYHZB6FCJMEETQZTZHWQIVLG26BPQ</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallet connection was smooth and straightforward.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recurring invoices for retainer work.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues at all.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A more detailed help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/29/2026 01:10:13</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jumoke Oyelaran</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jumoke5@gmail.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCJ2HRWZ25GUVTEDZYSU4QAQC74UXF5ZQNEJUBYY7YRYXUT4YA5UYINF</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moving between sections of the app was effortless.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A native mobile app.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add reporting tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/29/2026 10:30:45</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moyo Yusuf</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">moyo2@gmail.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GC25F7ML5AUYZ4I3UKZ2O5CRYRMWQELGCM5T2V3HHFXHEVKBKHYYMCSO</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payment reminders are a thoughtful feature.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice templates and customization.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No usability issues.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A short onboarding tutorial for new users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/29/2026 16:56:50</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lola Onwuka</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lola1@gmail.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDZXNG3AEIKOSQIQCN5J3G7OBFOCMLSTQ6UR4SSKRZN5KOYRO7YKYTRQ</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The interface is modern and easy to understand.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nil</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs. The experience was smooth overall.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for payment status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/30/2026 07:22:24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fatima Obi</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fatima2@gmail.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GASMYJWQ7YID66T6NHFVD534JM57FBQXNBNHLITBEVQ3JDVE2R7C5LCY</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The onboarding tour helped me get started quickly.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies in the future.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No usability issues.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A short onboarding tutorial for new users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/30/2026 09:11:02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temidayo Okocha</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temidayo.okocha@gmail.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAS57VHYXYXZBZ46ADDKRZKHWSHFROHV4QRAFE4KCPT77YBXRTZIPKCO</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallet connection was smooth and straightforward.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues during my testing.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maybe</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A short onboarding tutorial for new users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/31/2026 02:01:08</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Funmilayo Eze</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">funmilayo.eze@gmail.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAHE6GAQ5X3ZMZGMGDL5N7HZXYP2S3TLNSRWHIXDMRTSWENMBHXUODK6</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moving between sections of the app was effortless.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Team accounts for agencies.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor: the preview modal was slow to open once.</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maybe</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/31/2026 06:03:22</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Olawale Igwe</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">olawaleigwe@gmail.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBQXY27IDFX2FA7WQZJDVPWL7OXVDB2ZSIO2Q7H5TJRXH6J2PUXPB5QY</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The onboarding tour helped me get started quickly.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A quick product walkthrough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7/31/2026 12:40:08</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sade Akinwande</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sade6@gmail.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAYPSGJRN2MRCVY3RJCACXLWWK4K2UZP4UXCJ6HCBYEVMAMO7G7ZV6AX</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The activity page with on-chain proof is a nice touch.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for invoice updates.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No usability issues.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/1/2026 05:51:17</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seyi Oyelaran</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">seoyelaran@gmail.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBJ4KGUNTPAX7CVL3PXC6LOEDL5BGO6ZNGL2QPGOPHCS5I4NYTMQRLFB</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moving between sections of the app was effortless.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues during my testing.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maybe</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/1/2026 12:42:17</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ada Nwachukwu</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adanwachukwu@gmail.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDKEYHLUCVOT6VWWFBMP6VGXWR3OXMACH4QOKUJXTCDGFFAJOSRCVL76</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Receiving USDC straight to my wallet felt seamless.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies in the future.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/1/2026 21:17:35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rotimi Okocha</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rotimi.okocha@gmail.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBQLCPCEYTEMZLA44BDJMVKAYVHQWJ57FDKFG6CASTSB6PWPHBT4AWZE</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF export made sharing invoices very easy.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recurring invoices for retainer work.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Everything worked smoothly.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A short onboarding tutorial for new users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/2/2026 03:23:37</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chiamaka Olu</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chiamaka.olu@gmail.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GA2DLZELF45JYK2LO2LICBRPIQK72ZSXZYG6KTFYDTQ6BB4GUKUO7MTV</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The dashboard is clean and well organized.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nil</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I had to refresh once after connecting my wallet.</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nil</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/2/2026 15:42:25</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zainab Okeke</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">zaokeke@gmail.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAJZ4YFI5U6DZ4SYV5XD754VMIC7MPW7JZUXLS5OOGJR25C5SIGWC4AP</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payment reminders are a thoughtful feature.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">More reporting and analytics tools.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No usability issues.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add reporting tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/3/2026 00:22:44</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ada Okocha</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adaokocha@gmail.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBFC7D7CKYNSFBH5GSWJ54VEQZLA6RCC3YJY5B5OIXKMOAF77LV5USW6</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The activity page with on-chain proof is a nice touch.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for invoice updates.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues at all.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/3/2026 13:33:38</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temitope Akpan</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temitopeakpan@gmail.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDSB4LOO2XWBCLCTLVX7EWZ53NWBMGRS4ZCOBXMYBVLGDIONZ4MHWJOC</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dark mode looks clean and professional.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Everything worked smoothly.</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maybe</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/3/2026 16:17:43</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chinwe Igwe</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chinwe1@gmail.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GANYWN6EYRGMF6E7ZZKOP2UPB2QIYLMQ75HQN2S4Q2WNSVW2ULBD4EK7</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payment reminders are a thoughtful feature.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A quick product walkthrough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/4/2026 04:19:19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngozi Olawale</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ngozi7@gmail.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCMMAZEL67TMZVKQGISVMKD34SN4I4YDT4HCKSR4WPPTZ56UMA3G574Y</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Receiving USDC straight to my wallet felt seamless.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nil</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs. The experience was smooth overall.</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A short onboarding tutorial for new users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/4/2026 14:19:08</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Osagie Alabi</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">osagiealabi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCRI5DGWY3MPPDRTRW3SJ4VYZEE5JJE5RNOABU7LNIQRCBIS33GBRNSP</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The onboarding tour helped me get started quickly.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Team accounts for agencies.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs. The experience was smooth overall.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A more detailed help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/5/2026 00:31:50</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sade Okocha</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sade.okocha@gmail.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GD7Q3VYIS3WZ4WKNRJGKJY2ZQYMK2JOQT2VTTA2VEAQNW5MPYOBOBKMG</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The interface is modern and easy to understand.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nil</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs noticed.</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/5/2026 05:52:33</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Osagie Oyinlola</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">osagieoyinlola@gmail.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDOFPMNXJC4RXELNT4GWNJPFZKEBVEM5EI4YHK56RFKD2OTTUUMC4RF3</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The interface is modern and easy to understand.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for invoice updates.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add reporting tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/5/2026 20:53:06</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Funmilayo Gbadamosi</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">funmilayo3@gmail.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCCM37LKAL3EGOA6RXXYHMHSPSIQE4K6XAJSELTCZG2RY2ZTIA6SM3SE</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The one-click payment reminder is super useful.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies in the future.</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A more detailed help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/6/2026 02:48:47</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngozi Olu</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ngozi8@gmail.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GC74BSRWQKAII3SWK6OIPH24TU5QFCFL55KWOUMXTLDN2MO3OPF6C5M4</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moving between sections of the app was effortless.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for invoice updates.</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs. The experience was smooth overall.</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/6/2026 09:18:15</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emeka Olu</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emeka.olu@gmail.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCAU47PSRNEOGYWWNAPUH6PVBDARL4YC4CUJS3LJY6FO7SHPYQJRU6QL</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallet connection was smooth and straightforward.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">More reporting and analytics tools.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor: the preview modal was slow to open once.</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/6/2026 21:23:18</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngozi Nwosu</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ngnwosu@gmail.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBJMEROB7TPASM2L6H3PLU5AKY4SKYBCRJ62YG5TEUWNYTPOBWMT3KS7</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallet connection was smooth and straightforward.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recurring invoices for retainer work.</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I had to refresh once after connecting my wallet.</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A quick product walkthrough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/7/2026 10:23:55</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sade Okeke</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">saokeke@gmail.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBT34FWSESKTL34INHABUJOYEDBEZZ7MG3VWXSZHMTGXDEOOXXSU254Z</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The one-click payment reminder is super useful.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice templates and customization.</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I had to refresh once after connecting my wallet.</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add reporting tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/7/2026 15:47:28</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gbenga Okoro</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gbengaokoro@gmail.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCGTDSGFV2PJA46RSE54QSF7Y6IHSYVDKTAKJIBVE55GBBZAM5AJFGKX</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Creating invoices was simple and fast.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The dashboard took a few extra seconds to load once.</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A more detailed help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/8/2026 02:54:37</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makinwa Gbadamosi</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">makinwa.gbadamosi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDPIXUKBINF367BQSBBRJSX5HQEJJZGDO7KP3KKTZT3A3GA6D2QHWLNU</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The activity page with on-chain proof is a nice touch.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Team accounts for agencies.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faster loading on mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/8/2026 15:39:31</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Latifa Okoro</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">latifa9@gmail.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GBNYRUZ4KWUAWUN65R5TGYPXVWBLBNDNEBYPDLLLFJNRMZQDKFB367BA</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice history with search and filters is really handy.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Team accounts for agencies.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs noticed.</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maybe</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A more detailed help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/8/2026 20:36:13</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rahman Oyelaran</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rahmanoyelaran@gmail.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCM2T52RVOAWLKIDGIKGDCIOYJCRDJGGVBZPS6RCDSXW65TBT34BRWVF</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The one-click payment reminder is super useful.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice templates and customization.</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor: the preview modal was slow to open once.</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/9/2026 10:43:56</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chiamaka Kalu</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chkalu@gmail.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCLIXXFJLP7BWHPKZ2TLYFSNZYR4BMSAIYFQ4PK3YSMPGHAYMX4IZSLU</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dark mode looks clean and professional.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice templates and customization.</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No usability issues.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A quick product walkthrough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/9/2026 12:54:00</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emeka Balogun</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emeka.balogun@gmail.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDTIDFORIAZRVDJALTRMWOQD3DZRGSGLPZQK2CEQBICRGO5YXVD55YRD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Creating invoices was simple and fast.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">More reporting and analytics tools.</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I had to refresh once after connecting my wallet.</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for payment status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/10/2026 01:45:30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zara Oyinlola</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">zaoyinlola@gmail.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAYSME6QAMLBDM7ZRWBKERWXBPTVRZ357GNY5XACYXK5XKAMYKLOCLE3</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Receiving USDC straight to my wallet felt seamless.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A native mobile app.</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No issues during my testing.</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Email notifications for payment status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/10/2026 10:47:31</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chidimma Igwe</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chidimmaigwe@gmail.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GCOVX6LEFJMFID3J3BP64MTG7ZWGCTTTUUEETSWB5EPQXI57QNMBAF7L</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF export made sharing invoices very easy.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recurring invoices for retainer work.</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A more detailed help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/10/2026 21:24:32</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngozi Tella</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ngtella@gmail.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAJM57QAZVPP67546AB5FCELOPU7KG75RXNEYKRLWFMPU6GXTZNLE3TL</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Settlement was almost instant after my client paid.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice templates and customization.</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The dashboard took a few extra seconds to load once.</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice search and filtering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/11/2026 05:02:47</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temidayo Okeke</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temidayo.okeke@gmail.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GDF5HU2GOYTYE3KWONIRIPHDQMOJM2R3NB4HOU3GZHFYIRZAPBWCA4VJ</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The interface is modern and easy to understand.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Team accounts for agencies.</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs noticed.</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A quick product walkthrough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8/11/2026 17:39:02</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ada Adeyemi</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adadeyemi@gmail.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GC6ZXHGLV2AFDQR3Y6TVUBSMQJSUTFNBPGQU5H4YZNIJCSPD6J4G5EEJ</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testnet</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The pay link made it easy for my client to settle.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies in the future.</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No bugs. The experience was smooth overall.</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for more currencies.</t>
         </is>
       </c>
     </row>
@@ -719,7 +3569,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">60</t>
         </is>
       </c>
     </row>
@@ -731,7 +3581,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.3</t>
+          <t xml:space="preserve">5.23</t>
         </is>
       </c>
     </row>
@@ -743,7 +3593,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">60</t>
         </is>
       </c>
     </row>
@@ -755,7 +3605,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">52</t>
         </is>
       </c>
     </row>
@@ -779,7 +3629,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
     </row>
@@ -803,7 +3653,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10 18:23:23</t>
+          <t xml:space="preserve">2026-08-13 14:05:39</t>
         </is>
       </c>
     </row>

</xml_diff>